<commit_message>
changed the drivers visibility after consultation with Manick
</commit_message>
<xml_diff>
--- a/data/unsold_final.xlsx
+++ b/data/unsold_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - TVS Motor Company Ltd\LocaldriveD\All_VS_code_deployments\Revisit_model\P_revisits_V2\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tvshosur-my.sharepoint.com/personal/r_sivaarvind_tvsmotor_com/Documents/LocaldriveD/All_VS_code_deployments/Sales_model/Sivas_models/P_sales_newdigitalCP_event1_2_V5/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE952BF7-63E6-47B9-9611-7436439885B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{AE952BF7-63E6-47B9-9611-7436439885B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{956E72D9-03B1-4426-973C-A3D0D5659D6F}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{8CEA30C9-3F85-4132-BF40-CDBD4E738972}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{8CEA30C9-3F85-4132-BF40-CDBD4E738972}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="37">
   <si>
     <t>Opening month</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>TVS Emerald Auralis</t>
+  </si>
+  <si>
+    <t>TVS Emerald Altura</t>
   </si>
 </sst>
 </file>
@@ -569,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90DDB097-08BC-4120-90CA-A968FBECCF0D}">
-  <dimension ref="A1:J473"/>
+  <dimension ref="A1:J474"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" style="1" customWidth="1"/>
@@ -11136,6 +11139,29 @@
         <v>355</v>
       </c>
     </row>
+    <row r="474" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A474" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B474">
+        <v>2026</v>
+      </c>
+      <c r="C474" t="s">
+        <v>17</v>
+      </c>
+      <c r="D474" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E474">
+        <v>0</v>
+      </c>
+      <c r="F474" s="1">
+        <v>46173</v>
+      </c>
+      <c r="G474">
+        <v>975</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated unsold and cyclic for april to may26
</commit_message>
<xml_diff>
--- a/data/unsold_final.xlsx
+++ b/data/unsold_final.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tvshosur-my.sharepoint.com/personal/r_sivaarvind_tvsmotor_com/Documents/LocaldriveD/All_VS_code_deployments/Sales_model/Sivas_models/P_sales_newdigitalCP_event1_2_V5/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{AE952BF7-63E6-47B9-9611-7436439885B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{956E72D9-03B1-4426-973C-A3D0D5659D6F}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{AE952BF7-63E6-47B9-9611-7436439885B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{199A7FFF-DD5C-49F1-8BF5-577D4111BF20}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{8CEA30C9-3F85-4132-BF40-CDBD4E738972}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8CEA30C9-3F85-4132-BF40-CDBD4E738972}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="37">
   <si>
     <t>Opening month</t>
   </si>
@@ -572,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90DDB097-08BC-4120-90CA-A968FBECCF0D}">
-  <dimension ref="A1:J474"/>
+  <dimension ref="A1:J484"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" style="1" customWidth="1"/>
@@ -11162,6 +11162,236 @@
         <v>975</v>
       </c>
     </row>
+    <row r="475" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A475" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B475">
+        <v>2026</v>
+      </c>
+      <c r="C475" t="s">
+        <v>18</v>
+      </c>
+      <c r="D475" t="s">
+        <v>35</v>
+      </c>
+      <c r="E475">
+        <v>4</v>
+      </c>
+      <c r="F475" s="1">
+        <v>45970</v>
+      </c>
+      <c r="G475">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="476" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A476" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B476">
+        <v>2026</v>
+      </c>
+      <c r="C476" t="s">
+        <v>18</v>
+      </c>
+      <c r="D476" t="s">
+        <v>32</v>
+      </c>
+      <c r="E476">
+        <v>28</v>
+      </c>
+      <c r="F476" s="1">
+        <v>0</v>
+      </c>
+      <c r="G476">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="477" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A477" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B477">
+        <v>2026</v>
+      </c>
+      <c r="C477" t="s">
+        <v>18</v>
+      </c>
+      <c r="D477" t="s">
+        <v>23</v>
+      </c>
+      <c r="E477">
+        <v>4</v>
+      </c>
+      <c r="F477" s="1">
+        <v>44256</v>
+      </c>
+      <c r="G477">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="478" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A478" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B478">
+        <v>2026</v>
+      </c>
+      <c r="C478" t="s">
+        <v>18</v>
+      </c>
+      <c r="D478" t="s">
+        <v>28</v>
+      </c>
+      <c r="E478">
+        <v>11</v>
+      </c>
+      <c r="F478" s="1">
+        <v>45214</v>
+      </c>
+      <c r="G478">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="479" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A479" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B479">
+        <v>2026</v>
+      </c>
+      <c r="C479" t="s">
+        <v>18</v>
+      </c>
+      <c r="D479" t="s">
+        <v>29</v>
+      </c>
+      <c r="E479">
+        <v>1</v>
+      </c>
+      <c r="F479" s="1">
+        <v>44240</v>
+      </c>
+      <c r="G479">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="480" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A480" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B480">
+        <v>2026</v>
+      </c>
+      <c r="C480" t="s">
+        <v>18</v>
+      </c>
+      <c r="D480" t="s">
+        <v>33</v>
+      </c>
+      <c r="E480">
+        <v>158</v>
+      </c>
+      <c r="F480" s="1">
+        <v>45627</v>
+      </c>
+      <c r="G480">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="481" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A481" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B481">
+        <v>2026</v>
+      </c>
+      <c r="C481" t="s">
+        <v>18</v>
+      </c>
+      <c r="D481" t="s">
+        <v>30</v>
+      </c>
+      <c r="E481">
+        <v>1</v>
+      </c>
+      <c r="F481" s="1">
+        <v>45201</v>
+      </c>
+      <c r="G481">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="482" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A482" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B482">
+        <v>2026</v>
+      </c>
+      <c r="C482" t="s">
+        <v>18</v>
+      </c>
+      <c r="D482" t="s">
+        <v>34</v>
+      </c>
+      <c r="E482">
+        <v>154</v>
+      </c>
+      <c r="F482" s="1">
+        <v>45930</v>
+      </c>
+      <c r="G482">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="483" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A483" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B483">
+        <v>2026</v>
+      </c>
+      <c r="C483" t="s">
+        <v>18</v>
+      </c>
+      <c r="D483" t="s">
+        <v>31</v>
+      </c>
+      <c r="E483">
+        <v>42</v>
+      </c>
+      <c r="F483" s="1">
+        <v>45459</v>
+      </c>
+      <c r="G483">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="484" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A484" s="1">
+        <v>46143</v>
+      </c>
+      <c r="B484">
+        <v>2026</v>
+      </c>
+      <c r="C484" t="s">
+        <v>18</v>
+      </c>
+      <c r="D484" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E484">
+        <v>0</v>
+      </c>
+      <c r="F484" s="1">
+        <v>46173</v>
+      </c>
+      <c r="G484">
+        <v>975</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>